<commit_message>
MDL - Clase 7
</commit_message>
<xml_diff>
--- a/Deep Learning/Modelos de DL/Notebooks/MLP.xlsx
+++ b/Deep Learning/Modelos de DL/Notebooks/MLP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carrasco\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodrigobenitez/Documents/GitHub/ORT-AI/Deep Learning/Modelos de DL/Notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D15C256A-BC31-4387-BCEA-8ACCE293F3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6A5118-BDB2-6A46-993F-8302816DF227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{A2F18437-323D-4BF3-893B-852504B3BFD8}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17480" xr2:uid="{A2F18437-323D-4BF3-893B-852504B3BFD8}"/>
   </bookViews>
   <sheets>
     <sheet name="MLP" sheetId="2" r:id="rId1"/>
@@ -1079,13 +1079,13 @@
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1116,7 +1116,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1347,37 +1347,37 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>3.1440639679385738</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>2.1710974512080612</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>1.3132616875182228</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.66845964801328639</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.28733532511543075</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.11018460301110888</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>3.9953333162430306E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>1.4163456931505055E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>4.9791772043272986E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>1.7452233476729375E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>6.110660222530661E-4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1485,37 +1485,37 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>1.3132616875182228</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>1.0766366958882392</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.86589293718007532</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.68319717972663419</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.52926044903028424</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.40318604888545784</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.30266034739773889</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.22440559704717067</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.16472272508020849</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>0.11996196663434808</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.69314718055994529</c:v>
+                  <c:v>8.6836152153949631E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1623,37 +1623,37 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-0.18813419610827087</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.21428568568922335</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.56485035559375019</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.77978067624131064</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.81491910545668078</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.72220595506091767</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.5843626949492905</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.45106408285598681</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.33996419067652245</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.25335323225579048</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.1881223448878715</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2919,7 +2919,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -3236,26 +3236,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD13171B-11DC-4FF8-A9CD-73F8344D90F7}">
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.140625" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.1640625" customWidth="1"/>
     <col min="17" max="17" width="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.5" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="8" customFormat="1" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="8" customFormat="1" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -3302,7 +3302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" ht="19" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3311,38 +3311,38 @@
       </c>
       <c r="C2" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>-0.18813419610827087</v>
       </c>
       <c r="D2" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>0</v>
+        <v>3.5394475745305319E-2</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>10</v>
       </c>
       <c r="H2" s="9">
-        <v>0</v>
+        <v>-10.5</v>
       </c>
       <c r="I2" s="10">
-        <v>0</v>
+        <v>-3.4</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>12</v>
       </c>
       <c r="K2" s="11">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>15</v>
       </c>
       <c r="M2" s="13">
-        <v>0</v>
+        <v>-0.9</v>
       </c>
       <c r="N2" s="5" t="s">
         <v>18</v>
       </c>
       <c r="O2" s="15">
-        <v>0</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="Q2">
         <f>G12</f>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="R2" s="29">
         <f>J12</f>
-        <v>0.69314718055994529</v>
+        <v>3.1440639679385738</v>
       </c>
       <c r="S2">
         <f>Q2</f>
@@ -3358,17 +3358,17 @@
       </c>
       <c r="T2" s="30">
         <f>J13</f>
-        <v>0.69314718055994529</v>
+        <v>1.3132616875182228</v>
       </c>
       <c r="U2">
         <v>0</v>
       </c>
       <c r="V2" s="31">
         <f>L12</f>
-        <v>0</v>
+        <v>-0.18813419610827087</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" ht="19" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0.128</v>
       </c>
@@ -3377,23 +3377,23 @@
       </c>
       <c r="C3" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.32100180681171853</v>
       </c>
       <c r="D3" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>3.8025000000000003E-2</v>
+        <v>1.5876455319817635E-2</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="K3" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>16</v>
       </c>
       <c r="M3" s="14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q3">
         <f>G14</f>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="R3" s="29">
         <f>J14</f>
-        <v>0.69314718055994529</v>
+        <v>2.1710974512080612</v>
       </c>
       <c r="S3">
         <f t="shared" ref="S3:S12" si="0">Q3</f>
@@ -3409,17 +3409,17 @@
       </c>
       <c r="T3" s="30">
         <f>J15</f>
-        <v>0.69314718055994529</v>
+        <v>1.0766366958882392</v>
       </c>
       <c r="U3">
         <v>0.1</v>
       </c>
       <c r="V3" s="31">
         <f>L14</f>
-        <v>0</v>
+        <v>0.21428568568922335</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>0.24099999999999999</v>
       </c>
@@ -3428,11 +3428,11 @@
       </c>
       <c r="C4" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.6739254509958057</v>
       </c>
       <c r="D4" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>0.23522499999999999</v>
+        <v>3.5692826033968582E-2</v>
       </c>
       <c r="Q4">
         <f>G16</f>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="R4" s="29">
         <f>J16</f>
-        <v>0.69314718055994529</v>
+        <v>1.3132616875182228</v>
       </c>
       <c r="S4">
         <f t="shared" si="0"/>
@@ -3448,17 +3448,17 @@
       </c>
       <c r="T4" s="30">
         <f>J17</f>
-        <v>0.69314718055994529</v>
+        <v>0.86589293718007532</v>
       </c>
       <c r="U4">
         <v>0.2</v>
       </c>
       <c r="V4" s="31">
         <f>L16</f>
-        <v>0</v>
+        <v>0.56485035559375019</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>0.34200000000000003</v>
       </c>
@@ -3467,11 +3467,11 @@
       </c>
       <c r="C5" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.81537707946383686</v>
       </c>
       <c r="D5" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>0.71233599999999997</v>
+        <v>8.192715800195079E-4</v>
       </c>
       <c r="Q5">
         <f>G18</f>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="R5" s="29">
         <f>J18</f>
-        <v>0.69314718055994529</v>
+        <v>0.66845964801328639</v>
       </c>
       <c r="S5">
         <f t="shared" si="0"/>
@@ -3487,17 +3487,17 @@
       </c>
       <c r="T5" s="30">
         <f>J19</f>
-        <v>0.69314718055994529</v>
+        <v>0.68319717972663419</v>
       </c>
       <c r="U5">
         <v>0.3</v>
       </c>
       <c r="V5" s="31">
         <f>L18</f>
-        <v>0</v>
+        <v>0.77978067624131064</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" ht="19" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>0.501</v>
       </c>
@@ -3506,11 +3506,11 @@
       </c>
       <c r="C6" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.72093350071431572</v>
       </c>
       <c r="D6" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>1</v>
+        <v>7.7878111023566829E-2</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>3</v>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="R6" s="29">
         <f>J20</f>
-        <v>0.69314718055994529</v>
+        <v>0.28733532511543075</v>
       </c>
       <c r="S6">
         <f t="shared" si="0"/>
@@ -3532,17 +3532,17 @@
       </c>
       <c r="T6" s="30">
         <f>J21</f>
-        <v>0.69314718055994529</v>
+        <v>0.52926044903028424</v>
       </c>
       <c r="U6">
         <v>0.4</v>
       </c>
       <c r="V6" s="31">
         <f>L20</f>
-        <v>0</v>
+        <v>0.81491910545668078</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" ht="19" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0.627</v>
       </c>
@@ -3551,11 +3551,11 @@
       </c>
       <c r="C7" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.54676149463926427</v>
       </c>
       <c r="D7" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>0.84456100000000012</v>
+        <v>0.13856150487319452</v>
       </c>
       <c r="G7" t="s">
         <v>0</v>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="R7" s="29">
         <f>J22</f>
-        <v>0.69314718055994529</v>
+        <v>0.11018460301110888</v>
       </c>
       <c r="S7">
         <f t="shared" si="0"/>
@@ -3577,17 +3577,17 @@
       </c>
       <c r="T7" s="30">
         <f>J23</f>
-        <v>0.69314718055994529</v>
+        <v>0.40318604888545784</v>
       </c>
       <c r="U7">
         <v>0.5</v>
       </c>
       <c r="V7" s="31">
         <f>L22</f>
-        <v>0</v>
+        <v>0.72220595506091767</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" ht="19" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>0.82699999999999996</v>
       </c>
@@ -3596,11 +3596,11 @@
       </c>
       <c r="C8" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.31424733559817553</v>
       </c>
       <c r="D8" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>0.11764900000000002</v>
+        <v>8.2671571020394589E-4</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>9</v>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="R8" s="29">
         <f>J24</f>
-        <v>0.69314718055994529</v>
+        <v>3.9953333162430306E-2</v>
       </c>
       <c r="S8">
         <f t="shared" si="0"/>
@@ -3622,17 +3622,17 @@
       </c>
       <c r="T8" s="30">
         <f>J25</f>
-        <v>0.69314718055994529</v>
+        <v>0.30266034739773889</v>
       </c>
       <c r="U8">
         <v>0.6</v>
       </c>
       <c r="V8" s="31">
         <f>L24</f>
-        <v>0</v>
+        <v>0.5843626949492905</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>0.92500000000000004</v>
       </c>
@@ -3641,11 +3641,11 @@
       </c>
       <c r="C9" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.23520654662786217</v>
       </c>
       <c r="D9" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>3.4969E-2</v>
+        <v>2.3238711377842492E-3</v>
       </c>
       <c r="Q9">
         <f>G26</f>
@@ -3653,7 +3653,7 @@
       </c>
       <c r="R9" s="29">
         <f>J26</f>
-        <v>0.69314718055994529</v>
+        <v>1.4163456931505055E-2</v>
       </c>
       <c r="S9">
         <f t="shared" si="0"/>
@@ -3661,17 +3661,17 @@
       </c>
       <c r="T9" s="30">
         <f>J27</f>
-        <v>0.69314718055994529</v>
+        <v>0.22440559704717067</v>
       </c>
       <c r="U9">
         <v>0.7</v>
       </c>
       <c r="V9" s="31">
         <f>L26</f>
-        <v>0</v>
+        <v>0.45106408285598681</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1</v>
       </c>
@@ -3680,11 +3680,11 @@
       </c>
       <c r="C10" s="25">
         <f>LN(1+EXP(MLP[[#This Row],[x]]*$H$2+$K$2))*$M$2+LN(1+EXP(MLP[[#This Row],[x]]*$I$2+$K$3))*$M$3+$O$2</f>
-        <v>0</v>
+        <v>0.1881223448878715</v>
       </c>
       <c r="D10" s="25">
         <f>(MLP[[#This Row],[y_hat]]-MLP[[#This Row],[y]])^2</f>
-        <v>0</v>
+        <v>3.5390016646111272E-2</v>
       </c>
       <c r="Q10">
         <f>G28</f>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="R10" s="29">
         <f>J28</f>
-        <v>0.69314718055994529</v>
+        <v>4.9791772043272986E-3</v>
       </c>
       <c r="S10">
         <f t="shared" si="0"/>
@@ -3700,24 +3700,24 @@
       </c>
       <c r="T10" s="30">
         <f>J29</f>
-        <v>0.69314718055994529</v>
+        <v>0.16472272508020849</v>
       </c>
       <c r="U10">
         <v>0.8</v>
       </c>
       <c r="V10" s="31">
         <f>L28</f>
-        <v>0</v>
+        <v>0.33996419067652245</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="Q11">
         <f>G30</f>
         <v>0.9</v>
       </c>
       <c r="R11" s="29">
         <f>J30</f>
-        <v>0.69314718055994529</v>
+        <v>1.7452233476729375E-3</v>
       </c>
       <c r="S11">
         <f t="shared" si="0"/>
@@ -3725,25 +3725,25 @@
       </c>
       <c r="T11" s="30">
         <f>J31</f>
-        <v>0.69314718055994529</v>
+        <v>0.11996196663434808</v>
       </c>
       <c r="U11">
         <v>0.9</v>
       </c>
       <c r="V11" s="31">
         <f>L30</f>
-        <v>0</v>
+        <v>0.25335323225579048</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="C12" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="34">
+      <c r="D12" s="32">
         <f>AVERAGE(MLP[diff^2])</f>
-        <v>0.33141833333333337</v>
-      </c>
-      <c r="G12" s="32">
+        <v>3.8084805341107981E-2</v>
+      </c>
+      <c r="G12" s="34">
         <v>0</v>
       </c>
       <c r="H12" s="16">
@@ -3752,19 +3752,19 @@
       </c>
       <c r="I12" s="17">
         <f>H12+$K$2</f>
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="J12" s="22">
         <f t="shared" ref="J12:J33" si="1">LN(1+EXP(I12))</f>
-        <v>0.69314718055994529</v>
+        <v>3.1440639679385738</v>
       </c>
       <c r="K12" s="33">
         <f>J12*$M$2+J13*$M$3</f>
-        <v>0</v>
+        <v>-0.20313419610827088</v>
       </c>
       <c r="L12" s="33">
         <f>K12+$O$2</f>
-        <v>0</v>
+        <v>-0.18813419610827087</v>
       </c>
       <c r="Q12">
         <f>G32</f>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="R12" s="29">
         <f>J32</f>
-        <v>0.69314718055994529</v>
+        <v>6.110660222530661E-4</v>
       </c>
       <c r="S12">
         <f t="shared" si="0"/>
@@ -3780,472 +3780,455 @@
       </c>
       <c r="T12" s="30">
         <f>J33</f>
-        <v>0.69314718055994529</v>
+        <v>8.6836152153949631E-2</v>
       </c>
       <c r="U12">
         <v>1</v>
       </c>
       <c r="V12" s="31">
         <f>L32</f>
-        <v>0</v>
+        <v>0.1881223448878715</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G13" s="32"/>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="G13" s="34"/>
       <c r="H13" s="18">
         <f>$I$2*G12</f>
         <v>0</v>
       </c>
       <c r="I13" s="19">
         <f>H13+$K$3</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>1.3132616875182228</v>
       </c>
       <c r="K13" s="33"/>
       <c r="L13" s="33"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G14" s="32">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="G14" s="34">
         <v>0.1</v>
       </c>
       <c r="H14" s="16">
         <f>$H$2*G14</f>
-        <v>0</v>
+        <v>-1.05</v>
       </c>
       <c r="I14" s="17">
         <f>H14+$K$2</f>
-        <v>0</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="J14" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>2.1710974512080612</v>
       </c>
       <c r="K14" s="33">
         <f>J14*$M$2+J15*$M$3</f>
-        <v>0</v>
+        <v>0.19928568568922334</v>
       </c>
       <c r="L14" s="33">
         <f>K14+$O$2</f>
-        <v>0</v>
+        <v>0.21428568568922335</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G15" s="32"/>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="G15" s="34"/>
       <c r="H15" s="18">
         <f>$I$2*G14</f>
-        <v>0</v>
+        <v>-0.34</v>
       </c>
       <c r="I15" s="19">
         <f>H15+$K$3</f>
-        <v>0</v>
+        <v>0.65999999999999992</v>
       </c>
       <c r="J15" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>1.0766366958882392</v>
       </c>
       <c r="K15" s="33"/>
       <c r="L15" s="33"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G16" s="32">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="G16" s="34">
         <v>0.2</v>
       </c>
       <c r="H16" s="16">
         <f>$H$2*G16</f>
-        <v>0</v>
+        <v>-2.1</v>
       </c>
       <c r="I16" s="17">
         <f>H16+$K$2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>1.3132616875182228</v>
       </c>
       <c r="K16" s="33">
         <f>J16*$M$2+J17*$M$3</f>
-        <v>0</v>
+        <v>0.54985035559375017</v>
       </c>
       <c r="L16" s="33">
         <f>K16+$O$2</f>
-        <v>0</v>
+        <v>0.56485035559375019</v>
       </c>
     </row>
-    <row r="17" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G17" s="32"/>
+    <row r="17" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G17" s="34"/>
       <c r="H17" s="18">
         <f>$I$2*G16</f>
-        <v>0</v>
+        <v>-0.68</v>
       </c>
       <c r="I17" s="19">
         <f>H17+$K$3</f>
-        <v>0</v>
+        <v>0.31999999999999995</v>
       </c>
       <c r="J17" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.86589293718007532</v>
       </c>
       <c r="K17" s="33"/>
       <c r="L17" s="33"/>
     </row>
-    <row r="18" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G18" s="32">
+    <row r="18" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G18" s="34">
         <v>0.3</v>
       </c>
       <c r="H18" s="16">
         <f>$H$2*G18</f>
-        <v>0</v>
+        <v>-3.15</v>
       </c>
       <c r="I18" s="17">
         <f>H18+$K$2</f>
-        <v>0</v>
+        <v>-4.9999999999999822E-2</v>
       </c>
       <c r="J18" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.66845964801328639</v>
       </c>
       <c r="K18" s="33">
         <f>J18*$M$2+J19*$M$3</f>
-        <v>0</v>
+        <v>0.76478067624131063</v>
       </c>
       <c r="L18" s="33">
         <f>K18+$O$2</f>
-        <v>0</v>
+        <v>0.77978067624131064</v>
       </c>
     </row>
-    <row r="19" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G19" s="32"/>
+    <row r="19" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G19" s="34"/>
       <c r="H19" s="18">
         <f>$I$2*G18</f>
-        <v>0</v>
+        <v>-1.02</v>
       </c>
       <c r="I19" s="19">
         <f>H19+$K$3</f>
-        <v>0</v>
+        <v>-2.0000000000000018E-2</v>
       </c>
       <c r="J19" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.68319717972663419</v>
       </c>
       <c r="K19" s="33"/>
       <c r="L19" s="33"/>
     </row>
-    <row r="20" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G20" s="32">
+    <row r="20" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G20" s="34">
         <v>0.4</v>
       </c>
       <c r="H20" s="16">
         <f>$H$2*G20</f>
-        <v>0</v>
+        <v>-4.2</v>
       </c>
       <c r="I20" s="17">
         <f>H20+$K$2</f>
-        <v>0</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="J20" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.28733532511543075</v>
       </c>
       <c r="K20" s="33">
         <f>J20*$M$2+J21*$M$3</f>
-        <v>0</v>
+        <v>0.79991910545668077</v>
       </c>
       <c r="L20" s="33">
         <f>K20+$O$2</f>
-        <v>0</v>
+        <v>0.81491910545668078</v>
       </c>
     </row>
-    <row r="21" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G21" s="32"/>
+    <row r="21" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G21" s="34"/>
       <c r="H21" s="18">
         <f>$I$2*G20</f>
-        <v>0</v>
+        <v>-1.36</v>
       </c>
       <c r="I21" s="19">
         <f>H21+$K$3</f>
-        <v>0</v>
+        <v>-0.3600000000000001</v>
       </c>
       <c r="J21" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.52926044903028424</v>
       </c>
       <c r="K21" s="33"/>
       <c r="L21" s="33"/>
     </row>
-    <row r="22" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G22" s="32">
+    <row r="22" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G22" s="34">
         <v>0.5</v>
       </c>
       <c r="H22" s="16">
         <f>$H$2*G22</f>
-        <v>0</v>
+        <v>-5.25</v>
       </c>
       <c r="I22" s="17">
         <f>H22+$K$2</f>
-        <v>0</v>
+        <v>-2.15</v>
       </c>
       <c r="J22" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.11018460301110888</v>
       </c>
       <c r="K22" s="33">
         <f>J22*$M$2+J23*$M$3</f>
-        <v>0</v>
+        <v>0.70720595506091766</v>
       </c>
       <c r="L22" s="33">
         <f>K22+$O$2</f>
-        <v>0</v>
+        <v>0.72220595506091767</v>
       </c>
     </row>
-    <row r="23" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G23" s="32"/>
+    <row r="23" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G23" s="34"/>
       <c r="H23" s="18">
         <f>$I$2*G22</f>
-        <v>0</v>
+        <v>-1.7</v>
       </c>
       <c r="I23" s="19">
         <f>H23+$K$3</f>
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="J23" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.40318604888545784</v>
       </c>
       <c r="K23" s="33"/>
       <c r="L23" s="33"/>
     </row>
-    <row r="24" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G24" s="32">
+    <row r="24" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G24" s="34">
         <v>0.6</v>
       </c>
       <c r="H24" s="16">
         <f>$H$2*G24</f>
-        <v>0</v>
+        <v>-6.3</v>
       </c>
       <c r="I24" s="17">
         <f>H24+$K$2</f>
-        <v>0</v>
+        <v>-3.1999999999999997</v>
       </c>
       <c r="J24" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>3.9953333162430306E-2</v>
       </c>
       <c r="K24" s="33">
         <f>J24*$M$2+J25*$M$3</f>
-        <v>0</v>
+        <v>0.56936269494929048</v>
       </c>
       <c r="L24" s="33">
         <f>K24+$O$2</f>
-        <v>0</v>
+        <v>0.5843626949492905</v>
       </c>
     </row>
-    <row r="25" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G25" s="32"/>
+    <row r="25" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G25" s="34"/>
       <c r="H25" s="18">
         <f>$I$2*G24</f>
-        <v>0</v>
+        <v>-2.04</v>
       </c>
       <c r="I25" s="19">
         <f>H25+$K$3</f>
-        <v>0</v>
+        <v>-1.04</v>
       </c>
       <c r="J25" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.30266034739773889</v>
       </c>
       <c r="K25" s="33"/>
       <c r="L25" s="33"/>
     </row>
-    <row r="26" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G26" s="32">
+    <row r="26" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G26" s="34">
         <v>0.7</v>
       </c>
       <c r="H26" s="16">
         <f>$H$2*G26</f>
-        <v>0</v>
+        <v>-7.35</v>
       </c>
       <c r="I26" s="17">
         <f>H26+$K$2</f>
-        <v>0</v>
+        <v>-4.25</v>
       </c>
       <c r="J26" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>1.4163456931505055E-2</v>
       </c>
       <c r="K26" s="33">
         <f>J26*$M$2+J27*$M$3</f>
-        <v>0</v>
+        <v>0.4360640828559868</v>
       </c>
       <c r="L26" s="33">
         <f>K26+$O$2</f>
-        <v>0</v>
+        <v>0.45106408285598681</v>
       </c>
     </row>
-    <row r="27" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G27" s="32"/>
+    <row r="27" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G27" s="34"/>
       <c r="H27" s="18">
         <f>$I$2*G26</f>
-        <v>0</v>
+        <v>-2.38</v>
       </c>
       <c r="I27" s="19">
         <f>H27+$K$3</f>
-        <v>0</v>
+        <v>-1.38</v>
       </c>
       <c r="J27" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.22440559704717067</v>
       </c>
       <c r="K27" s="33"/>
       <c r="L27" s="33"/>
     </row>
-    <row r="28" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G28" s="32">
+    <row r="28" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G28" s="34">
         <v>0.8</v>
       </c>
       <c r="H28" s="16">
         <f>$H$2*G28</f>
-        <v>0</v>
+        <v>-8.4</v>
       </c>
       <c r="I28" s="17">
         <f>H28+$K$2</f>
-        <v>0</v>
+        <v>-5.3000000000000007</v>
       </c>
       <c r="J28" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>4.9791772043272986E-3</v>
       </c>
       <c r="K28" s="33">
         <f>J28*$M$2+J29*$M$3</f>
-        <v>0</v>
+        <v>0.32496419067652244</v>
       </c>
       <c r="L28" s="33">
         <f>K28+$O$2</f>
-        <v>0</v>
+        <v>0.33996419067652245</v>
       </c>
     </row>
-    <row r="29" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G29" s="32"/>
+    <row r="29" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G29" s="34"/>
       <c r="H29" s="18">
         <f>$I$2*G28</f>
-        <v>0</v>
+        <v>-2.72</v>
       </c>
       <c r="I29" s="19">
         <f>H29+$K$3</f>
-        <v>0</v>
+        <v>-1.7200000000000002</v>
       </c>
       <c r="J29" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.16472272508020849</v>
       </c>
       <c r="K29" s="33"/>
       <c r="L29" s="33"/>
     </row>
-    <row r="30" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G30" s="32">
+    <row r="30" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G30" s="34">
         <v>0.9</v>
       </c>
       <c r="H30" s="16">
         <f>$H$2*G30</f>
-        <v>0</v>
+        <v>-9.4500000000000011</v>
       </c>
       <c r="I30" s="17">
         <f>H30+$K$2</f>
-        <v>0</v>
+        <v>-6.3500000000000014</v>
       </c>
       <c r="J30" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>1.7452233476729375E-3</v>
       </c>
       <c r="K30" s="33">
         <f>J30*$M$2+J31*$M$3</f>
-        <v>0</v>
+        <v>0.2383532322557905</v>
       </c>
       <c r="L30" s="33">
         <f>K30+$O$2</f>
-        <v>0</v>
+        <v>0.25335323225579048</v>
       </c>
     </row>
-    <row r="31" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G31" s="32"/>
+    <row r="31" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G31" s="34"/>
       <c r="H31" s="18">
         <f>$I$2*G30</f>
-        <v>0</v>
+        <v>-3.06</v>
       </c>
       <c r="I31" s="19">
         <f>H31+$K$3</f>
-        <v>0</v>
+        <v>-2.06</v>
       </c>
       <c r="J31" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>0.11996196663434808</v>
       </c>
       <c r="K31" s="33"/>
       <c r="L31" s="33"/>
     </row>
-    <row r="32" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G32" s="32">
+    <row r="32" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G32" s="34">
         <v>1</v>
       </c>
       <c r="H32" s="20">
         <f>$H$2*G32</f>
-        <v>0</v>
+        <v>-10.5</v>
       </c>
       <c r="I32" s="21">
         <f>H32+$K$2</f>
-        <v>0</v>
+        <v>-7.4</v>
       </c>
       <c r="J32" s="22">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>6.110660222530661E-4</v>
       </c>
       <c r="K32" s="33">
         <f>J32*$M$2+J33*$M$3</f>
-        <v>0</v>
+        <v>0.17312234488787151</v>
       </c>
       <c r="L32" s="33">
         <f>K32+$O$2</f>
-        <v>0</v>
+        <v>0.1881223448878715</v>
       </c>
     </row>
-    <row r="33" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G33" s="32"/>
+    <row r="33" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G33" s="34"/>
       <c r="H33" s="18">
         <f>$I$2*G32</f>
-        <v>0</v>
+        <v>-3.4</v>
       </c>
       <c r="I33" s="19">
         <f>H33+$K$3</f>
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="J33" s="23">
         <f t="shared" si="1"/>
-        <v>0.69314718055994529</v>
+        <v>8.6836152153949631E-2</v>
       </c>
       <c r="K33" s="33"/>
       <c r="L33" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="K24:K25"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="L12:L13"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="G20:G21"/>
     <mergeCell ref="G32:G33"/>
     <mergeCell ref="L14:L15"/>
     <mergeCell ref="L16:L17"/>
@@ -4262,6 +4245,23 @@
     <mergeCell ref="K30:K31"/>
     <mergeCell ref="K32:K33"/>
     <mergeCell ref="G22:G23"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="K16:K17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>